<commit_message>
data (The Eyes of the Dragon)
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/code/projects/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48FAF91B-4635-C74F-A7BF-0F728429C49D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DD25A5E-7B51-524F-AE69-BDB9AF3621C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11880" yWindow="760" windowWidth="15440" windowHeight="19000" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="-20" yWindow="680" windowWidth="15420" windowHeight="18980" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="226">
   <si>
     <t>book_id</t>
   </si>
@@ -710,6 +710,9 @@
   </si>
   <si>
     <t>Ines Cagnati</t>
+  </si>
+  <si>
+    <t>The Eyes of the Dragon</t>
   </si>
 </sst>
 </file>
@@ -1112,7 +1115,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FE0100-68F1-984E-9C9C-2E858B800C9D}">
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
@@ -2236,6 +2239,44 @@
         <v>46226</v>
       </c>
     </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>225</v>
+      </c>
+      <c r="C30" t="s">
+        <v>140</v>
+      </c>
+      <c r="D30" t="s">
+        <v>80</v>
+      </c>
+      <c r="E30">
+        <v>1984</v>
+      </c>
+      <c r="F30" t="s">
+        <v>130</v>
+      </c>
+      <c r="G30">
+        <v>326</v>
+      </c>
+      <c r="H30" s="11">
+        <v>105474</v>
+      </c>
+      <c r="I30" t="s">
+        <v>104</v>
+      </c>
+      <c r="J30" t="s">
+        <v>81</v>
+      </c>
+      <c r="K30" s="7">
+        <v>46227</v>
+      </c>
+      <c r="L30" s="7">
+        <v>46229</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2243,7 +2284,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E7A9E8-5203-EC4D-9951-9FF3806CB4E8}">
-  <dimension ref="A1:I283"/>
+  <dimension ref="A1:I293"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -7675,7 +7716,7 @@
     </row>
     <row r="259" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A259">
-        <f t="shared" ref="A259:A283" si="4">ROW() - 1</f>
+        <f t="shared" ref="A259:A293" si="4">ROW() - 1</f>
         <v>258</v>
       </c>
       <c r="B259">
@@ -8196,6 +8237,216 @@
       </c>
       <c r="F283" s="6">
         <v>2.3842592592592592E-2</v>
+      </c>
+    </row>
+    <row r="284" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A284">
+        <f t="shared" si="4"/>
+        <v>283</v>
+      </c>
+      <c r="B284">
+        <v>29</v>
+      </c>
+      <c r="C284" s="3">
+        <v>46227.950694444444</v>
+      </c>
+      <c r="D284" t="s">
+        <v>63</v>
+      </c>
+      <c r="E284" t="s">
+        <v>63</v>
+      </c>
+      <c r="F284" s="6">
+        <v>1.8576388888888889E-2</v>
+      </c>
+    </row>
+    <row r="285" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A285">
+        <f t="shared" si="4"/>
+        <v>284</v>
+      </c>
+      <c r="B285">
+        <v>29</v>
+      </c>
+      <c r="C285" s="3">
+        <v>46228.426388888889</v>
+      </c>
+      <c r="D285" t="s">
+        <v>63</v>
+      </c>
+      <c r="E285" t="s">
+        <v>63</v>
+      </c>
+      <c r="F285" s="6">
+        <v>1.4699074074074074E-2</v>
+      </c>
+    </row>
+    <row r="286" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A286">
+        <f t="shared" si="4"/>
+        <v>285</v>
+      </c>
+      <c r="B286">
+        <v>29</v>
+      </c>
+      <c r="C286" s="3">
+        <v>46228.63958333333</v>
+      </c>
+      <c r="D286" t="s">
+        <v>63</v>
+      </c>
+      <c r="E286" t="s">
+        <v>63</v>
+      </c>
+      <c r="F286" s="6">
+        <v>2.2928240740740742E-2</v>
+      </c>
+    </row>
+    <row r="287" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A287">
+        <f t="shared" si="4"/>
+        <v>286</v>
+      </c>
+      <c r="B287">
+        <v>29</v>
+      </c>
+      <c r="C287" s="3">
+        <v>46228.706250000003</v>
+      </c>
+      <c r="D287" t="s">
+        <v>63</v>
+      </c>
+      <c r="E287" t="s">
+        <v>63</v>
+      </c>
+      <c r="F287" s="6">
+        <v>2.5104166666666667E-2</v>
+      </c>
+    </row>
+    <row r="288" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A288">
+        <f t="shared" si="4"/>
+        <v>287</v>
+      </c>
+      <c r="B288">
+        <v>29</v>
+      </c>
+      <c r="C288" s="3">
+        <v>46228.775694444441</v>
+      </c>
+      <c r="D288" t="s">
+        <v>63</v>
+      </c>
+      <c r="E288" t="s">
+        <v>63</v>
+      </c>
+      <c r="F288" s="6">
+        <v>2.1770833333333333E-2</v>
+      </c>
+    </row>
+    <row r="289" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A289">
+        <f t="shared" si="4"/>
+        <v>288</v>
+      </c>
+      <c r="B289">
+        <v>29</v>
+      </c>
+      <c r="C289" s="3">
+        <v>46228.820138888892</v>
+      </c>
+      <c r="D289" t="s">
+        <v>63</v>
+      </c>
+      <c r="E289" t="s">
+        <v>63</v>
+      </c>
+      <c r="F289" s="6">
+        <v>2.1134259259259259E-2</v>
+      </c>
+    </row>
+    <row r="290" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A290">
+        <f t="shared" si="4"/>
+        <v>289</v>
+      </c>
+      <c r="B290">
+        <v>29</v>
+      </c>
+      <c r="C290" s="3">
+        <v>46228.931944444441</v>
+      </c>
+      <c r="D290" t="s">
+        <v>63</v>
+      </c>
+      <c r="E290" t="s">
+        <v>63</v>
+      </c>
+      <c r="F290" s="6">
+        <v>1.8148148148148149E-2</v>
+      </c>
+    </row>
+    <row r="291" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A291">
+        <f t="shared" si="4"/>
+        <v>290</v>
+      </c>
+      <c r="B291">
+        <v>29</v>
+      </c>
+      <c r="C291" s="3">
+        <v>46229.418055555558</v>
+      </c>
+      <c r="D291" t="s">
+        <v>63</v>
+      </c>
+      <c r="E291" t="s">
+        <v>63</v>
+      </c>
+      <c r="F291" s="6">
+        <v>2.2199074074074072E-2</v>
+      </c>
+    </row>
+    <row r="292" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A292">
+        <f t="shared" si="4"/>
+        <v>291</v>
+      </c>
+      <c r="B292">
+        <v>29</v>
+      </c>
+      <c r="C292" s="3">
+        <v>46229.490277777775</v>
+      </c>
+      <c r="D292" t="s">
+        <v>63</v>
+      </c>
+      <c r="E292" t="s">
+        <v>63</v>
+      </c>
+      <c r="F292" s="6">
+        <v>2.5173611111111112E-2</v>
+      </c>
+    </row>
+    <row r="293" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A293">
+        <f t="shared" si="4"/>
+        <v>292</v>
+      </c>
+      <c r="B293">
+        <v>29</v>
+      </c>
+      <c r="C293" s="3">
+        <v>46229.529861111114</v>
+      </c>
+      <c r="D293" t="s">
+        <v>63</v>
+      </c>
+      <c r="E293" t="s">
+        <v>63</v>
+      </c>
+      <c r="F293" s="6">
+        <v>6.4467592592592588E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data (Soldiers & Sailors)
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/dev/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BF3B255-482C-E840-B17C-22B119190074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C412A9D1-F915-B246-BADB-27533A59D3A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="15420" windowHeight="18980" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="27540" windowHeight="18980" activeTab="2" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="253">
   <si>
     <t>book_id</t>
   </si>
@@ -785,6 +785,15 @@
   </si>
   <si>
     <t>Light Verse</t>
+  </si>
+  <si>
+    <t>Soldiers &amp; Sailors</t>
+  </si>
+  <si>
+    <t>Terrence Holt</t>
+  </si>
+  <si>
+    <t>supernatural</t>
   </si>
 </sst>
 </file>
@@ -1187,7 +1196,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FE0100-68F1-984E-9C9C-2E858B800C9D}">
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
@@ -2387,6 +2396,44 @@
         <v>46236</v>
       </c>
     </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>250</v>
+      </c>
+      <c r="C32" t="s">
+        <v>251</v>
+      </c>
+      <c r="D32" t="s">
+        <v>252</v>
+      </c>
+      <c r="E32">
+        <v>2026</v>
+      </c>
+      <c r="F32" t="s">
+        <v>16</v>
+      </c>
+      <c r="G32">
+        <v>412</v>
+      </c>
+      <c r="H32" s="11">
+        <v>133625</v>
+      </c>
+      <c r="I32" t="s">
+        <v>105</v>
+      </c>
+      <c r="J32" t="s">
+        <v>67</v>
+      </c>
+      <c r="K32" s="7">
+        <v>46239</v>
+      </c>
+      <c r="L32" s="7">
+        <v>46183</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2394,7 +2441,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E7A9E8-5203-EC4D-9951-9FF3806CB4E8}">
-  <dimension ref="A1:I303"/>
+  <dimension ref="A1:I316"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -7826,7 +7873,7 @@
     </row>
     <row r="259" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A259">
-        <f t="shared" ref="A259:A303" si="4">ROW() - 1</f>
+        <f t="shared" ref="A259:A316" si="4">ROW() - 1</f>
         <v>258</v>
       </c>
       <c r="B259">
@@ -8767,6 +8814,279 @@
       </c>
       <c r="F303" s="6">
         <v>2.2534722222222223E-2</v>
+      </c>
+    </row>
+    <row r="304" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A304">
+        <f t="shared" si="4"/>
+        <v>303</v>
+      </c>
+      <c r="B304">
+        <v>31</v>
+      </c>
+      <c r="C304" s="3">
+        <v>46239.493055555555</v>
+      </c>
+      <c r="D304">
+        <v>3</v>
+      </c>
+      <c r="E304">
+        <v>26</v>
+      </c>
+      <c r="F304" s="6">
+        <v>1.7696759259259259E-2</v>
+      </c>
+    </row>
+    <row r="305" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A305">
+        <f t="shared" si="4"/>
+        <v>304</v>
+      </c>
+      <c r="B305">
+        <v>31</v>
+      </c>
+      <c r="C305" s="3">
+        <v>46239.772222222222</v>
+      </c>
+      <c r="D305">
+        <v>26</v>
+      </c>
+      <c r="E305">
+        <v>50</v>
+      </c>
+      <c r="F305" s="6">
+        <v>1.6851851851851851E-2</v>
+      </c>
+    </row>
+    <row r="306" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A306">
+        <f t="shared" si="4"/>
+        <v>305</v>
+      </c>
+      <c r="B306">
+        <v>31</v>
+      </c>
+      <c r="C306" s="3">
+        <v>46240.534722222219</v>
+      </c>
+      <c r="D306">
+        <v>50</v>
+      </c>
+      <c r="E306">
+        <v>84</v>
+      </c>
+      <c r="F306" s="6">
+        <v>2.2928240740740742E-2</v>
+      </c>
+    </row>
+    <row r="307" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A307">
+        <f t="shared" si="4"/>
+        <v>306</v>
+      </c>
+      <c r="B307">
+        <v>31</v>
+      </c>
+      <c r="C307" s="3">
+        <v>46240.788194444445</v>
+      </c>
+      <c r="D307">
+        <v>84</v>
+      </c>
+      <c r="E307">
+        <v>87</v>
+      </c>
+      <c r="F307" s="6">
+        <v>2.5231481481481481E-3</v>
+      </c>
+    </row>
+    <row r="308" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A308">
+        <f t="shared" si="4"/>
+        <v>307</v>
+      </c>
+      <c r="B308">
+        <v>31</v>
+      </c>
+      <c r="C308" s="3">
+        <v>46240.806944444441</v>
+      </c>
+      <c r="D308">
+        <v>87</v>
+      </c>
+      <c r="E308">
+        <v>125</v>
+      </c>
+      <c r="F308" s="6">
+        <v>2.4212962962962964E-2</v>
+      </c>
+    </row>
+    <row r="309" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A309">
+        <f t="shared" si="4"/>
+        <v>308</v>
+      </c>
+      <c r="B309">
+        <v>31</v>
+      </c>
+      <c r="C309" s="3">
+        <v>46242.006249999999</v>
+      </c>
+      <c r="D309">
+        <v>125</v>
+      </c>
+      <c r="E309">
+        <v>161</v>
+      </c>
+      <c r="F309" s="6">
+        <v>2.326388888888889E-2</v>
+      </c>
+    </row>
+    <row r="310" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A310">
+        <f t="shared" si="4"/>
+        <v>309</v>
+      </c>
+      <c r="B310">
+        <v>31</v>
+      </c>
+      <c r="C310" s="3">
+        <v>46242.917361111111</v>
+      </c>
+      <c r="D310">
+        <v>161</v>
+      </c>
+      <c r="E310">
+        <v>196</v>
+      </c>
+      <c r="F310" s="6">
+        <v>2.6666666666666668E-2</v>
+      </c>
+    </row>
+    <row r="311" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A311">
+        <f t="shared" si="4"/>
+        <v>310</v>
+      </c>
+      <c r="B311">
+        <v>31</v>
+      </c>
+      <c r="C311" s="3">
+        <v>46243.597222222219</v>
+      </c>
+      <c r="D311">
+        <v>196</v>
+      </c>
+      <c r="E311">
+        <v>228</v>
+      </c>
+      <c r="F311" s="6">
+        <v>2.1238425925925924E-2</v>
+      </c>
+    </row>
+    <row r="312" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A312">
+        <f t="shared" si="4"/>
+        <v>311</v>
+      </c>
+      <c r="B312">
+        <v>31</v>
+      </c>
+      <c r="C312" s="3">
+        <v>46243.736805555556</v>
+      </c>
+      <c r="D312">
+        <v>228</v>
+      </c>
+      <c r="E312">
+        <v>256</v>
+      </c>
+      <c r="F312" s="6">
+        <v>1.7592592592592594E-2</v>
+      </c>
+    </row>
+    <row r="313" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A313">
+        <f t="shared" si="4"/>
+        <v>312</v>
+      </c>
+      <c r="B313">
+        <v>31</v>
+      </c>
+      <c r="C313" s="3">
+        <v>46243.820138888892</v>
+      </c>
+      <c r="D313">
+        <v>256</v>
+      </c>
+      <c r="E313">
+        <v>270</v>
+      </c>
+      <c r="F313" s="6">
+        <v>9.0277777777777769E-3</v>
+      </c>
+    </row>
+    <row r="314" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A314">
+        <f t="shared" si="4"/>
+        <v>313</v>
+      </c>
+      <c r="B314">
+        <v>31</v>
+      </c>
+      <c r="C314" s="3">
+        <v>46243.98541666667</v>
+      </c>
+      <c r="D314">
+        <v>270</v>
+      </c>
+      <c r="E314">
+        <v>314</v>
+      </c>
+      <c r="F314" s="6">
+        <v>2.7071759259259261E-2</v>
+      </c>
+    </row>
+    <row r="315" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A315">
+        <f t="shared" si="4"/>
+        <v>314</v>
+      </c>
+      <c r="B315">
+        <v>31</v>
+      </c>
+      <c r="C315" s="3">
+        <v>46244.524305555555</v>
+      </c>
+      <c r="D315">
+        <v>314</v>
+      </c>
+      <c r="E315">
+        <v>353</v>
+      </c>
+      <c r="F315" s="6">
+        <v>2.4618055555555556E-2</v>
+      </c>
+    </row>
+    <row r="316" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A316">
+        <f t="shared" si="4"/>
+        <v>315</v>
+      </c>
+      <c r="B316">
+        <v>31</v>
+      </c>
+      <c r="C316" s="3">
+        <v>46244.906944444447</v>
+      </c>
+      <c r="D316">
+        <v>353</v>
+      </c>
+      <c r="E316">
+        <v>415</v>
+      </c>
+      <c r="F316" s="6">
+        <v>3.90625E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data (Crossing The Wine-Dark Sea)
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/dev/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C412A9D1-F915-B246-BADB-27533A59D3A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAEC6D80-2D25-884F-B2DB-8224AC0D0DF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="27540" windowHeight="18980" activeTab="2" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
+    <workbookView xWindow="-20" yWindow="680" windowWidth="14260" windowHeight="18980" activeTab="1" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
   <sheets>
     <sheet name="books" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="256">
   <si>
     <t>book_id</t>
   </si>
@@ -794,6 +794,15 @@
   </si>
   <si>
     <t>supernatural</t>
+  </si>
+  <si>
+    <t>Crossing The Wine-Dark Sea</t>
+  </si>
+  <si>
+    <t>Emily Wilson</t>
+  </si>
+  <si>
+    <t>nonfiction</t>
   </si>
 </sst>
 </file>
@@ -1196,11 +1205,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FE0100-68F1-984E-9C9C-2E858B800C9D}">
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.33203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -2434,6 +2443,44 @@
         <v>46183</v>
       </c>
     </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>253</v>
+      </c>
+      <c r="C33" t="s">
+        <v>254</v>
+      </c>
+      <c r="D33" t="s">
+        <v>255</v>
+      </c>
+      <c r="E33">
+        <v>2026</v>
+      </c>
+      <c r="F33" t="s">
+        <v>16</v>
+      </c>
+      <c r="G33">
+        <v>263</v>
+      </c>
+      <c r="H33" s="11">
+        <v>65523</v>
+      </c>
+      <c r="I33" t="s">
+        <v>104</v>
+      </c>
+      <c r="J33" t="s">
+        <v>67</v>
+      </c>
+      <c r="K33" s="7">
+        <v>46245</v>
+      </c>
+      <c r="L33" s="7">
+        <v>46248</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2441,7 +2488,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E7A9E8-5203-EC4D-9951-9FF3806CB4E8}">
-  <dimension ref="A1:I316"/>
+  <dimension ref="A1:I327"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -7873,7 +7920,7 @@
     </row>
     <row r="259" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A259">
-        <f t="shared" ref="A259:A316" si="4">ROW() - 1</f>
+        <f t="shared" ref="A259:A322" si="4">ROW() - 1</f>
         <v>258</v>
       </c>
       <c r="B259">
@@ -9087,6 +9134,237 @@
       </c>
       <c r="F316" s="6">
         <v>3.90625E-2</v>
+      </c>
+    </row>
+    <row r="317" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A317">
+        <f t="shared" si="4"/>
+        <v>316</v>
+      </c>
+      <c r="B317">
+        <v>32</v>
+      </c>
+      <c r="C317" s="3">
+        <v>46245.974305555559</v>
+      </c>
+      <c r="D317">
+        <v>1</v>
+      </c>
+      <c r="E317">
+        <v>27</v>
+      </c>
+      <c r="F317" s="6">
+        <v>1.9733796296296298E-2</v>
+      </c>
+    </row>
+    <row r="318" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A318">
+        <f t="shared" si="4"/>
+        <v>317</v>
+      </c>
+      <c r="B318">
+        <v>32</v>
+      </c>
+      <c r="C318" s="3">
+        <v>46246.438194444447</v>
+      </c>
+      <c r="D318">
+        <v>27</v>
+      </c>
+      <c r="E318">
+        <v>53</v>
+      </c>
+      <c r="F318" s="6">
+        <v>1.5486111111111112E-2</v>
+      </c>
+    </row>
+    <row r="319" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A319">
+        <f t="shared" si="4"/>
+        <v>318</v>
+      </c>
+      <c r="B319">
+        <v>32</v>
+      </c>
+      <c r="C319" s="3">
+        <v>46246.574999999997</v>
+      </c>
+      <c r="D319">
+        <v>53</v>
+      </c>
+      <c r="E319">
+        <v>81</v>
+      </c>
+      <c r="F319" s="6">
+        <v>1.7800925925925925E-2</v>
+      </c>
+    </row>
+    <row r="320" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A320">
+        <f t="shared" si="4"/>
+        <v>319</v>
+      </c>
+      <c r="B320">
+        <v>32</v>
+      </c>
+      <c r="C320" s="3">
+        <v>46246.92083333333</v>
+      </c>
+      <c r="D320">
+        <v>81</v>
+      </c>
+      <c r="E320">
+        <v>113</v>
+      </c>
+      <c r="F320" s="6">
+        <v>2.0925925925925924E-2</v>
+      </c>
+    </row>
+    <row r="321" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A321">
+        <f t="shared" si="4"/>
+        <v>320</v>
+      </c>
+      <c r="B321">
+        <v>32</v>
+      </c>
+      <c r="C321" s="3">
+        <v>46247.741666666669</v>
+      </c>
+      <c r="D321">
+        <v>113</v>
+      </c>
+      <c r="E321">
+        <v>132</v>
+      </c>
+      <c r="F321" s="6">
+        <v>1.2881944444444444E-2</v>
+      </c>
+    </row>
+    <row r="322" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A322">
+        <f t="shared" si="4"/>
+        <v>321</v>
+      </c>
+      <c r="B322">
+        <v>32</v>
+      </c>
+      <c r="C322" s="3">
+        <v>46247.775000000001</v>
+      </c>
+      <c r="D322">
+        <v>132</v>
+      </c>
+      <c r="E322">
+        <v>147</v>
+      </c>
+      <c r="F322" s="6">
+        <v>8.2060185185185187E-3</v>
+      </c>
+    </row>
+    <row r="323" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A323">
+        <f t="shared" ref="A323:A327" si="5">ROW() - 1</f>
+        <v>322</v>
+      </c>
+      <c r="B323">
+        <v>32</v>
+      </c>
+      <c r="C323" s="3">
+        <v>46247.827777777777</v>
+      </c>
+      <c r="D323">
+        <v>147</v>
+      </c>
+      <c r="E323">
+        <v>164</v>
+      </c>
+      <c r="F323" s="6">
+        <v>1.1226851851851852E-2</v>
+      </c>
+    </row>
+    <row r="324" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A324">
+        <f t="shared" si="5"/>
+        <v>323</v>
+      </c>
+      <c r="B324">
+        <v>32</v>
+      </c>
+      <c r="C324" s="3">
+        <v>46247.949305555558</v>
+      </c>
+      <c r="D324">
+        <v>164</v>
+      </c>
+      <c r="E324">
+        <v>181</v>
+      </c>
+      <c r="F324" s="6">
+        <v>1.4247685185185184E-2</v>
+      </c>
+    </row>
+    <row r="325" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A325">
+        <f t="shared" si="5"/>
+        <v>324</v>
+      </c>
+      <c r="B325">
+        <v>32</v>
+      </c>
+      <c r="C325" s="3">
+        <v>46248.494444444441</v>
+      </c>
+      <c r="D325">
+        <v>181</v>
+      </c>
+      <c r="E325">
+        <v>216</v>
+      </c>
+      <c r="F325" s="6">
+        <v>2.2789351851851852E-2</v>
+      </c>
+    </row>
+    <row r="326" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A326">
+        <f t="shared" si="5"/>
+        <v>325</v>
+      </c>
+      <c r="B326">
+        <v>32</v>
+      </c>
+      <c r="C326" s="3">
+        <v>46248.549305555556</v>
+      </c>
+      <c r="D326">
+        <v>216</v>
+      </c>
+      <c r="E326">
+        <v>258</v>
+      </c>
+      <c r="F326" s="6">
+        <v>2.1388888888888888E-2</v>
+      </c>
+    </row>
+    <row r="327" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A327">
+        <f t="shared" si="5"/>
+        <v>326</v>
+      </c>
+      <c r="B327">
+        <v>32</v>
+      </c>
+      <c r="C327" s="3">
+        <v>46248.584722222222</v>
+      </c>
+      <c r="D327">
+        <v>258</v>
+      </c>
+      <c r="E327">
+        <v>263</v>
+      </c>
+      <c r="F327" s="6">
+        <v>2.627314814814815E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data (The Absolute at Large)
</commit_message>
<xml_diff>
--- a/data/reading-data.xlsx
+++ b/data/reading-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericmoore/dev/reading-analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB9FA6DB-771F-DF4D-8699-A8876A92BAC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C3B85E3-286E-524B-B379-B0FB851EA9F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="15100" windowHeight="18960" xr2:uid="{FD2DF24A-B0C8-8B40-8EA1-ACF2DA714EAB}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="265">
   <si>
     <t>book_id</t>
   </si>
@@ -824,6 +824,12 @@
   </si>
   <si>
     <t>Contents</t>
+  </si>
+  <si>
+    <t>The Absolute at Large</t>
+  </si>
+  <si>
+    <t>Karel Capek</t>
   </si>
 </sst>
 </file>
@@ -1229,7 +1235,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56FE0100-68F1-984E-9C9C-2E858B800C9D}">
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
@@ -2543,6 +2549,44 @@
         <v>46259</v>
       </c>
     </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>263</v>
+      </c>
+      <c r="C35" t="s">
+        <v>264</v>
+      </c>
+      <c r="D35" t="s">
+        <v>15</v>
+      </c>
+      <c r="E35">
+        <v>1927</v>
+      </c>
+      <c r="F35" t="s">
+        <v>14</v>
+      </c>
+      <c r="G35">
+        <v>242</v>
+      </c>
+      <c r="H35" s="11">
+        <v>50164</v>
+      </c>
+      <c r="I35" t="s">
+        <v>102</v>
+      </c>
+      <c r="J35" t="s">
+        <v>65</v>
+      </c>
+      <c r="K35" s="7">
+        <v>46260</v>
+      </c>
+      <c r="L35" s="7">
+        <v>46263</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2550,7 +2594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E7A9E8-5203-EC4D-9951-9FF3806CB4E8}">
-  <dimension ref="A1:H340"/>
+  <dimension ref="A1:H348"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.5" bestFit="1" customWidth="1"/>
@@ -8340,6 +8384,142 @@
       </c>
       <c r="E340" s="6">
         <v>1.6307870370370372E-2</v>
+      </c>
+    </row>
+    <row r="341" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A341">
+        <v>34</v>
+      </c>
+      <c r="B341" s="3">
+        <v>46260.493750000001</v>
+      </c>
+      <c r="C341">
+        <v>1</v>
+      </c>
+      <c r="D341">
+        <v>34</v>
+      </c>
+      <c r="E341" s="6">
+        <v>1.2662037037037038E-2</v>
+      </c>
+    </row>
+    <row r="342" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A342">
+        <v>34</v>
+      </c>
+      <c r="B342" s="3">
+        <v>46261.380555555559</v>
+      </c>
+      <c r="C342">
+        <v>34</v>
+      </c>
+      <c r="D342">
+        <v>60</v>
+      </c>
+      <c r="E342" s="6">
+        <v>1.0659722222222221E-2</v>
+      </c>
+    </row>
+    <row r="343" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A343">
+        <v>34</v>
+      </c>
+      <c r="B343" s="3">
+        <v>46261.582638888889</v>
+      </c>
+      <c r="C343">
+        <v>60</v>
+      </c>
+      <c r="D343">
+        <v>103</v>
+      </c>
+      <c r="E343" s="6">
+        <v>1.9629629629629629E-2</v>
+      </c>
+    </row>
+    <row r="344" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A344">
+        <v>34</v>
+      </c>
+      <c r="B344" s="3">
+        <v>46261.926388888889</v>
+      </c>
+      <c r="C344">
+        <v>103</v>
+      </c>
+      <c r="D344">
+        <v>138</v>
+      </c>
+      <c r="E344" s="6">
+        <v>1.8055555555555554E-2</v>
+      </c>
+    </row>
+    <row r="345" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A345">
+        <v>34</v>
+      </c>
+      <c r="B345" s="3">
+        <v>46262.441666666666</v>
+      </c>
+      <c r="C345">
+        <v>138</v>
+      </c>
+      <c r="D345">
+        <v>177</v>
+      </c>
+      <c r="E345" s="6">
+        <v>1.7037037037037038E-2</v>
+      </c>
+    </row>
+    <row r="346" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A346">
+        <v>34</v>
+      </c>
+      <c r="B346" s="3">
+        <v>46262.638888888891</v>
+      </c>
+      <c r="C346">
+        <v>177</v>
+      </c>
+      <c r="D346">
+        <v>189</v>
+      </c>
+      <c r="E346" s="6">
+        <v>6.3078703703703708E-3</v>
+      </c>
+    </row>
+    <row r="347" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A347">
+        <v>34</v>
+      </c>
+      <c r="B347" s="3">
+        <v>46262.896527777775</v>
+      </c>
+      <c r="C347">
+        <v>189</v>
+      </c>
+      <c r="D347">
+        <v>216</v>
+      </c>
+      <c r="E347" s="6">
+        <v>1.3634259259259259E-2</v>
+      </c>
+    </row>
+    <row r="348" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A348">
+        <v>34</v>
+      </c>
+      <c r="B348" s="3">
+        <v>46263.434027777781</v>
+      </c>
+      <c r="C348">
+        <v>216</v>
+      </c>
+      <c r="D348">
+        <v>242</v>
+      </c>
+      <c r="E348" s="6">
+        <v>9.1550925925925931E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>